<commit_message>
fixing a few bugs, change levels
</commit_message>
<xml_diff>
--- a/Src/Assets/StreamingAssets/Common/Tables/Tables/Levels.xlsx
+++ b/Src/Assets/StreamingAssets/Common/Tables/Tables/Levels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CCA\Src\Assets\StreamingAssets\Common\Tables\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6247C4EC-EC8E-4121-BA6E-53C15E5AA14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC35383-6887-4925-B254-DEB5AF804F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Character" sheetId="2" r:id="rId1"/>
@@ -1366,19 +1366,11 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>["Intimidation","Void Servant","Devour the Stars","Morphing Remains"]</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
     <t>["Charge"]</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>["Time Reversal"]</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
-    <t>["Cocooning"]</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
@@ -2002,6 +1994,48 @@
       <t>]</t>
     </r>
     <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>["</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Time Fasting</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>"]</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>["Time Distortion","Void Servant","Devouring Stars","Morphing Remain"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -3226,13 +3260,13 @@
         <v>2</v>
       </c>
       <c r="E1" s="36" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="F1" s="22" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="36" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="H1" s="22" t="s">
         <v>8</v>
@@ -3297,7 +3331,7 @@
         <v>249</v>
       </c>
       <c r="M2" s="26" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N2" s="26" t="s">
         <v>356</v>
@@ -3343,7 +3377,7 @@
         <v>12</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N3" s="11" t="s">
         <v>356</v>
@@ -3387,7 +3421,7 @@
         <v>12</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N4" s="7" t="s">
         <v>356</v>
@@ -3433,7 +3467,7 @@
         <v>12</v>
       </c>
       <c r="M5" s="16" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N5" s="11" t="s">
         <v>356</v>
@@ -3477,10 +3511,10 @@
         <v>249</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
@@ -3507,7 +3541,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="29" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>11</v>
@@ -3520,10 +3554,10 @@
         <v>7</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N7" s="29" t="s">
         <v>357</v>
@@ -3567,7 +3601,7 @@
         <v>249</v>
       </c>
       <c r="M8" s="33" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N8" s="33" t="s">
         <v>358</v>
@@ -3597,7 +3631,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>16</v>
@@ -3616,7 +3650,7 @@
         <v>12</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N9" s="11" t="s">
         <v>356</v>
@@ -3643,7 +3677,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="32" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="H10" s="32" t="s">
         <v>16</v>
@@ -3662,7 +3696,7 @@
         <v>12</v>
       </c>
       <c r="M10" s="32" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N10" s="32" t="s">
         <v>356</v>
@@ -3709,7 +3743,7 @@
         <v>12</v>
       </c>
       <c r="M11" s="11" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N11" s="11" t="s">
         <v>356</v>
@@ -3753,7 +3787,7 @@
         <v>12</v>
       </c>
       <c r="M12" s="32" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N12" s="32" t="s">
         <v>356</v>
@@ -3771,7 +3805,7 @@
         <v>Skunk Chieftain</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>224</v>
@@ -3802,7 +3836,7 @@
         <v>354</v>
       </c>
       <c r="M13" s="11" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N13" s="11" t="s">
         <v>359</v>
@@ -3846,10 +3880,10 @@
         <v>249</v>
       </c>
       <c r="M14" s="33" t="s">
-        <v>417</v>
-      </c>
-      <c r="N14" s="33" t="s">
-        <v>360</v>
+        <v>415</v>
+      </c>
+      <c r="N14" s="32" t="s">
+        <v>490</v>
       </c>
       <c r="O14" s="33"/>
       <c r="P14" s="33"/>
@@ -3895,10 +3929,10 @@
         <v>245</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N15" s="29" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3941,10 +3975,10 @@
         <v>12</v>
       </c>
       <c r="M16" s="32" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N16" s="33" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="O16" s="32"/>
       <c r="P16" s="32"/>
@@ -3962,7 +3996,7 @@
         <v>101</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>232</v>
@@ -3990,10 +4024,10 @@
         <v>12</v>
       </c>
       <c r="M17" s="11" t="s">
-        <v>417</v>
-      </c>
-      <c r="N17" s="29" t="s">
-        <v>363</v>
+        <v>415</v>
+      </c>
+      <c r="N17" s="11" t="s">
+        <v>489</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4029,10 +4063,10 @@
         <v>12</v>
       </c>
       <c r="M18" s="32" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N18" s="33" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="O18" s="32"/>
       <c r="P18" s="32"/>
@@ -4076,7 +4110,7 @@
         <v>12</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N19" s="11" t="s">
         <v>356</v>
@@ -4117,13 +4151,13 @@
         <v>2</v>
       </c>
       <c r="L20" s="33" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="M20" s="32" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N20" s="33" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="O20" s="32"/>
       <c r="P20" s="32"/>
@@ -4150,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>11</v>
@@ -4169,10 +4203,10 @@
         <v>354</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N21" s="29" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4215,10 +4249,10 @@
         <v>12</v>
       </c>
       <c r="M22" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N22" s="53" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="O22" s="34"/>
       <c r="P22" s="34"/>
@@ -4264,10 +4298,10 @@
         <v>249</v>
       </c>
       <c r="M23" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N23" s="29" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="O23" s="29"/>
       <c r="P23" s="29"/>
@@ -4313,7 +4347,7 @@
         <v>249</v>
       </c>
       <c r="M24" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N24" s="34" t="s">
         <v>356</v>
@@ -4360,10 +4394,10 @@
         <v>249</v>
       </c>
       <c r="M25" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N25" s="29" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="O25" s="29"/>
       <c r="P25" s="29"/>
@@ -4407,7 +4441,7 @@
         <v>12</v>
       </c>
       <c r="M26" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N26" s="34" t="s">
         <v>356</v>
@@ -4454,10 +4488,10 @@
         <v>249</v>
       </c>
       <c r="M27" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N27" s="29" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="O27" s="29"/>
       <c r="P27" s="29"/>
@@ -4503,7 +4537,7 @@
         <v>12</v>
       </c>
       <c r="M28" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N28" s="34" t="s">
         <v>356</v>
@@ -4552,7 +4586,7 @@
         <v>249</v>
       </c>
       <c r="M29" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N29" s="29" t="s">
         <v>356</v>
@@ -4601,7 +4635,7 @@
         <v>249</v>
       </c>
       <c r="M30" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N30" s="34" t="s">
         <v>356</v>
@@ -4648,10 +4682,10 @@
         <v>249</v>
       </c>
       <c r="M31" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N31" s="29" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="O31" s="29"/>
       <c r="P31" s="29"/>
@@ -4678,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="53" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="H32" s="34" t="s">
         <v>11</v>
@@ -4697,10 +4731,10 @@
         <v>249</v>
       </c>
       <c r="M32" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N32" s="53" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="O32" s="34"/>
       <c r="P32" s="34"/>
@@ -4727,7 +4761,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="29" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="H33" s="29" t="s">
         <v>11</v>
@@ -4746,10 +4780,10 @@
         <v>249</v>
       </c>
       <c r="M33" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N33" s="29" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="O33" s="29"/>
       <c r="P33" s="29"/>
@@ -4776,7 +4810,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="34" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="H34" s="34" t="s">
         <v>11</v>
@@ -4795,10 +4829,10 @@
         <v>12</v>
       </c>
       <c r="M34" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N34" s="53" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="O34" s="34"/>
       <c r="P34" s="34"/>
@@ -4844,10 +4878,10 @@
         <v>249</v>
       </c>
       <c r="M35" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N35" s="29" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="O35" s="29"/>
       <c r="P35" s="29"/>
@@ -4891,10 +4925,10 @@
         <v>249</v>
       </c>
       <c r="M36" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N36" s="53" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="O36" s="34"/>
       <c r="P36" s="34"/>
@@ -4938,10 +4972,10 @@
         <v>249</v>
       </c>
       <c r="M37" s="29" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N37" s="29" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="O37" s="29"/>
       <c r="P37" s="29"/>
@@ -4985,10 +5019,10 @@
         <v>249</v>
       </c>
       <c r="M38" s="37" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N38" s="37" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="O38" s="37"/>
       <c r="P38" s="37"/>
@@ -5034,7 +5068,7 @@
         <v>12</v>
       </c>
       <c r="M39" s="11" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N39" s="29" t="s">
         <v>356</v>
@@ -5078,10 +5112,10 @@
         <v>249</v>
       </c>
       <c r="M40" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N40" s="39" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="O40" s="39"/>
       <c r="P40" s="39"/>
@@ -5127,10 +5161,10 @@
         <v>249</v>
       </c>
       <c r="M41" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N41" s="38" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="O41" s="38"/>
       <c r="P41" s="38"/>
@@ -5176,10 +5210,10 @@
         <v>249</v>
       </c>
       <c r="M42" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N42" s="39" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="O42" s="39"/>
       <c r="P42" s="39"/>
@@ -5222,13 +5256,13 @@
         <v>2</v>
       </c>
       <c r="L43" s="38" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="M43" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N43" s="38" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="O43" s="38"/>
       <c r="P43" s="38"/>
@@ -5258,7 +5292,7 @@
         <v>241</v>
       </c>
       <c r="H44" s="39" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="I44" s="39" t="s">
         <v>11</v>
@@ -5274,10 +5308,10 @@
         <v>249</v>
       </c>
       <c r="M44" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N44" s="39" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="O44" s="39"/>
       <c r="P44" s="39"/>
@@ -5320,13 +5354,13 @@
         <v>3</v>
       </c>
       <c r="L45" s="38" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="M45" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N45" s="38" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="O45" s="38"/>
       <c r="P45" s="38"/>
@@ -5372,10 +5406,10 @@
         <v>249</v>
       </c>
       <c r="M46" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N46" s="39" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="O46" s="39"/>
       <c r="P46" s="39"/>
@@ -5421,10 +5455,10 @@
         <v>249</v>
       </c>
       <c r="M47" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N47" s="38" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="O47" s="38"/>
       <c r="P47" s="38"/>
@@ -5470,10 +5504,10 @@
         <v>249</v>
       </c>
       <c r="M48" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N48" s="39" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="O48" s="39"/>
       <c r="P48" s="39"/>
@@ -5519,10 +5553,10 @@
         <v>249</v>
       </c>
       <c r="M49" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N49" s="38" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="O49" s="38"/>
       <c r="P49" s="38"/>
@@ -5568,10 +5602,10 @@
         <v>249</v>
       </c>
       <c r="M50" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N50" s="39" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="O50" s="39"/>
       <c r="P50" s="39"/>
@@ -5615,10 +5649,10 @@
         <v>249</v>
       </c>
       <c r="M51" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N51" s="38" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="O51" s="38"/>
       <c r="P51" s="38"/>
@@ -5660,10 +5694,10 @@
         <v>249</v>
       </c>
       <c r="M52" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N52" s="39" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="O52" s="39"/>
       <c r="P52" s="39"/>
@@ -5705,10 +5739,10 @@
         <v>249</v>
       </c>
       <c r="M53" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N53" s="38" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="O53" s="38"/>
       <c r="P53" s="38"/>
@@ -5752,10 +5786,10 @@
         <v>249</v>
       </c>
       <c r="M54" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N54" s="39" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="O54" s="39"/>
       <c r="P54" s="39"/>
@@ -5799,10 +5833,10 @@
         <v>249</v>
       </c>
       <c r="M55" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N55" s="38" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="O55" s="38"/>
       <c r="P55" s="38"/>
@@ -5845,13 +5879,13 @@
         <v>8</v>
       </c>
       <c r="L56" s="39" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="M56" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N56" s="39" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="O56" s="39"/>
       <c r="P56" s="39"/>
@@ -5897,10 +5931,10 @@
         <v>249</v>
       </c>
       <c r="M57" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N57" s="38" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="O57" s="38"/>
       <c r="P57" s="38"/>
@@ -5946,10 +5980,10 @@
         <v>249</v>
       </c>
       <c r="M58" s="39" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N58" s="39" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="O58" s="39"/>
       <c r="P58" s="39"/>
@@ -5987,10 +6021,10 @@
         <v>12</v>
       </c>
       <c r="M59" s="11" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N59" s="29" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="60" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6027,10 +6061,10 @@
         <v>249</v>
       </c>
       <c r="M60" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N60" s="41" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="O60" s="41"/>
       <c r="P60" s="41"/>
@@ -6072,10 +6106,10 @@
         <v>249</v>
       </c>
       <c r="M61" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N61" s="38" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="O61" s="38"/>
       <c r="P61" s="38"/>
@@ -6117,10 +6151,10 @@
         <v>249</v>
       </c>
       <c r="M62" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N62" s="41" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="O62" s="41"/>
       <c r="P62" s="41"/>
@@ -6160,10 +6194,10 @@
         <v>249</v>
       </c>
       <c r="M63" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N63" s="38" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="O63" s="38"/>
       <c r="P63" s="38"/>
@@ -6203,10 +6237,10 @@
         <v>249</v>
       </c>
       <c r="M64" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N64" s="41" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="O64" s="41"/>
       <c r="P64" s="41"/>
@@ -6246,10 +6280,10 @@
         <v>249</v>
       </c>
       <c r="M65" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N65" s="38" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="O65" s="38"/>
       <c r="P65" s="38"/>
@@ -6289,10 +6323,10 @@
         <v>249</v>
       </c>
       <c r="M66" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N66" s="41" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="O66" s="41"/>
       <c r="P66" s="41"/>
@@ -6332,10 +6366,10 @@
         <v>249</v>
       </c>
       <c r="M67" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N67" s="38" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="O67" s="38"/>
       <c r="P67" s="38"/>
@@ -6375,10 +6409,10 @@
         <v>249</v>
       </c>
       <c r="M68" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N68" s="41" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="O68" s="41"/>
       <c r="P68" s="41"/>
@@ -6418,10 +6452,10 @@
         <v>249</v>
       </c>
       <c r="M69" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N69" s="38" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="O69" s="38"/>
       <c r="P69" s="38"/>
@@ -6461,10 +6495,10 @@
         <v>249</v>
       </c>
       <c r="M70" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N70" s="41" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="O70" s="41"/>
       <c r="P70" s="41"/>
@@ -6506,10 +6540,10 @@
         <v>249</v>
       </c>
       <c r="M71" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N71" s="38" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="O71" s="38"/>
       <c r="P71" s="38"/>
@@ -6549,10 +6583,10 @@
         <v>249</v>
       </c>
       <c r="M72" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N72" s="41" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="O72" s="41"/>
       <c r="P72" s="41"/>
@@ -6594,10 +6628,10 @@
         <v>249</v>
       </c>
       <c r="M73" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N73" s="38" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="O73" s="38"/>
       <c r="P73" s="38"/>
@@ -6641,10 +6675,10 @@
         <v>249</v>
       </c>
       <c r="M74" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N74" s="41" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="O74" s="41"/>
       <c r="P74" s="41"/>
@@ -6688,10 +6722,10 @@
         <v>249</v>
       </c>
       <c r="M75" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N75" s="38" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="O75" s="38"/>
       <c r="P75" s="38"/>
@@ -6730,13 +6764,13 @@
         <v>13</v>
       </c>
       <c r="L76" s="41" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="M76" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N76" s="41" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="O76" s="41"/>
       <c r="P76" s="41"/>
@@ -6776,10 +6810,10 @@
         <v>249</v>
       </c>
       <c r="M77" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N77" s="38" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="O77" s="38"/>
       <c r="P77" s="38"/>
@@ -6821,10 +6855,10 @@
         <v>249</v>
       </c>
       <c r="M78" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N78" s="41" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="O78" s="41"/>
       <c r="P78" s="41"/>
@@ -6864,10 +6898,10 @@
         <v>249</v>
       </c>
       <c r="M79" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N79" s="38" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="O79" s="38"/>
       <c r="P79" s="38"/>
@@ -6907,10 +6941,10 @@
         <v>249</v>
       </c>
       <c r="M80" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N80" s="41" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="O80" s="41"/>
       <c r="P80" s="41"/>
@@ -6947,13 +6981,13 @@
         <v>28</v>
       </c>
       <c r="L81" s="38" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="M81" s="38" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N81" s="38" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="O81" s="38"/>
       <c r="P81" s="38"/>
@@ -6961,14 +6995,14 @@
     </row>
     <row r="82" spans="1:17" ht="13.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="41" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="B82" s="41" t="str">
         <f>A82</f>
         <v>Counter-Blade</v>
       </c>
       <c r="C82" s="41" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D82" s="41" t="s">
         <v>227</v>
@@ -6995,10 +7029,10 @@
         <v>249</v>
       </c>
       <c r="M82" s="41" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="N82" s="41" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="O82" s="41"/>
       <c r="P82" s="41"/>
@@ -7250,7 +7284,7 @@
         <v>29</v>
       </c>
       <c r="J1" s="56" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>30</v>
@@ -7262,10 +7296,10 @@
         <v>32</v>
       </c>
       <c r="N1" s="22" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="O1" s="22" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -7294,7 +7328,7 @@
         <v>314</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="J2" s="26" t="s">
         <v>314</v>
@@ -7340,10 +7374,10 @@
         <v>314</v>
       </c>
       <c r="I3" s="27" t="s">
+        <v>434</v>
+      </c>
+      <c r="J3" s="27" t="s">
         <v>436</v>
-      </c>
-      <c r="J3" s="27" t="s">
-        <v>438</v>
       </c>
       <c r="K3" s="16">
         <v>0</v>
@@ -7389,7 +7423,7 @@
         <v>314</v>
       </c>
       <c r="I4" s="26" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>314</v>
@@ -7429,16 +7463,16 @@
         <v>39</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="H5" s="16" t="s">
         <v>314</v>
       </c>
       <c r="I5" s="27" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="J5" s="16" t="s">
         <v>314</v>
@@ -7490,7 +7524,7 @@
         <v>11</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="K6" s="6">
         <v>1</v>
@@ -7499,7 +7533,7 @@
         <v>4</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="N6" s="6" t="str">
         <f t="shared" si="1"/>
@@ -7536,10 +7570,10 @@
         <v>314</v>
       </c>
       <c r="I7" s="27" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="J7" s="27" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="K7" s="16">
         <v>1</v>
@@ -7588,7 +7622,7 @@
         <v>42</v>
       </c>
       <c r="J8" s="52" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="K8" s="61">
         <v>1</v>
@@ -7597,7 +7631,7 @@
         <v>5</v>
       </c>
       <c r="M8" s="52" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="N8" s="52" t="str">
         <f t="shared" si="1"/>
@@ -7625,7 +7659,7 @@
         <v>281</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>314</v>
@@ -7634,10 +7668,10 @@
         <v>314</v>
       </c>
       <c r="I9" s="57" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="K9" s="27">
         <v>2</v>
@@ -7677,13 +7711,13 @@
         <v>310</v>
       </c>
       <c r="G10" s="66" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="H10" s="52" t="s">
         <v>314</v>
       </c>
       <c r="I10" s="52" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="J10" s="52" t="s">
         <v>314</v>
@@ -7732,10 +7766,10 @@
         <v>314</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="K11" s="27">
         <v>3</v>
@@ -7781,10 +7815,10 @@
         <v>314</v>
       </c>
       <c r="I12" s="66" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="J12" s="52" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="K12" s="61">
         <v>3</v>
@@ -7830,10 +7864,10 @@
         <v>314</v>
       </c>
       <c r="I13" s="27" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="J13" s="27" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="K13" s="16">
         <v>3</v>
@@ -7879,10 +7913,10 @@
         <v>314</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="J14" s="33" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="K14" s="33">
         <v>4</v>
@@ -7928,10 +7962,10 @@
         <v>314</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="K15" s="16">
         <v>4</v>
@@ -7980,7 +8014,7 @@
         <v>11</v>
       </c>
       <c r="J16" s="33" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="K16" s="33">
         <v>5</v>
@@ -8026,10 +8060,10 @@
         <v>314</v>
       </c>
       <c r="I17" s="27" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="J17" s="27" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="K17" s="16">
         <v>5</v>
@@ -8075,10 +8109,10 @@
         <v>314</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="J18" s="33" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="K18" s="33">
         <v>5</v>
@@ -8127,7 +8161,7 @@
         <v>314</v>
       </c>
       <c r="J19" s="27" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K19" s="16">
         <v>6</v>
@@ -8173,10 +8207,10 @@
         <v>314</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="J20" s="39" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="K20" s="39">
         <v>6</v>
@@ -8222,7 +8256,7 @@
         <v>314</v>
       </c>
       <c r="I21" s="27" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="J21" s="16" t="s">
         <v>314</v>
@@ -8271,10 +8305,10 @@
         <v>314</v>
       </c>
       <c r="I22" s="39" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="J22" s="39" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="K22" s="39">
         <v>6</v>
@@ -8323,7 +8357,7 @@
         <v>314</v>
       </c>
       <c r="J23" s="27" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="K23" s="16">
         <v>7</v>
@@ -8372,7 +8406,7 @@
         <v>314</v>
       </c>
       <c r="J24" s="39" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="K24" s="39">
         <v>8</v>
@@ -8470,7 +8504,7 @@
         <v>314</v>
       </c>
       <c r="J26" s="41" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="K26" s="41">
         <v>9</v>
@@ -8516,7 +8550,7 @@
         <v>314</v>
       </c>
       <c r="I27" s="27" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="J27" s="16" t="s">
         <v>314</v>
@@ -8559,7 +8593,7 @@
         <v>345</v>
       </c>
       <c r="G28" s="67" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="H28" s="41" t="s">
         <v>314</v>
@@ -8568,7 +8602,7 @@
         <v>11</v>
       </c>
       <c r="J28" s="41" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="K28" s="41">
         <v>10</v>
@@ -8608,7 +8642,7 @@
         <v>346</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="H29" s="16" t="s">
         <v>314</v>
@@ -8617,7 +8651,7 @@
         <v>11</v>
       </c>
       <c r="J29" s="27" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="K29" s="16">
         <v>11</v>
@@ -8657,7 +8691,7 @@
         <v>347</v>
       </c>
       <c r="G30" s="67" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="H30" s="41" t="s">
         <v>314</v>
@@ -8666,7 +8700,7 @@
         <v>11</v>
       </c>
       <c r="J30" s="41" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="K30" s="41">
         <v>12</v>
@@ -8706,7 +8740,7 @@
         <v>348</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="H31" s="16" t="s">
         <v>314</v>
@@ -8715,7 +8749,7 @@
         <v>11</v>
       </c>
       <c r="J31" s="27" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="K31" s="16">
         <v>12</v>

</xml_diff>